<commit_message>
Model the 10 CCU room sensors as orphans (assumption QNL-025)
The user directed these be treated as orphans, not assumed onto the register
CCUs that happen to share those rooms. Each tag is the sensor itself (a point),
so it is typed as its measurement class (brick:Relative_Humidity_Sensor /
brick:Temperature_Sensor), made brick:isPartOf entity:HVAC, given its timeseries
and unit, and NO rec:locatedIn - like the other orphans.

All 10 are in the Selected sheet and the historian. IO cross-check stays clean
(0 E-IO-1). Assumption log: QNL-025 added, QNL-024 revised down to the remaining
68 building/system-level tags whose parent still needs the client's direction.
Total ontology 8,378 rows. Row validator 554 IFC-empty + 7 accepted E-FEED-1 /
7 W-GR-2. Tests pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L1CU23wNWRi3FVm37EG2eh
</commit_message>
<xml_diff>
--- a/projects/QNL/QNL_Assumption_Log.xlsx
+++ b/projects/QNL/QNL_Assumption_Log.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1510,12 +1510,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>78 system/aggregate telemetry tags (CHW plant instrumentation 21, electrical metering 24, DX group/staging 11, CCU room sensors 10, misc 12)</t>
+          <t>68 system/aggregate telemetry tags (CHW plant instrumentation 21, electrical metering 24, DX group/staging 11, misc 12)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>In the historian and Selected sheet under a family prefix, but each is a single building- or system-level measurement, not an equipment unit (e.g. CHW_BldgAvgSupTemp, ELEC_MFM_MVP1, DX_RP21 staging, CCU_AVServerRmHumd)</t>
+          <t>In the historian and Selected sheet under a family prefix, but each is a single building- or system-level measurement, not tied to any register unit (e.g. CHW_BldgAvgSupTemp, ELEC_MFM_MVP1, DX_RP21 staging, TotalEnergy)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1525,12 +1525,59 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>These are points that need a parent entity - the chilled-water loop/system, the electrical system, or specific units - which the sources do not settle. Modelling them as standalone equipment would invent units that do not exist. Held for the client to direct where they attach.</t>
+          <t>These are points whose equipment parent is unknown, or building-level points with no equipment. Per the client, such points either attach to their equipment or, if none, to the building - to be confirmed per group before modelling. Held pending that direction.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>QNL-025</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>10 CCU room sensors (CCU_AVServerRm/MDFRm/QTelRm/ServerRm Humd &amp; Temp)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Selected + historian, named under the CCU prefix but not tied to any register CCU unit</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Modelled each as its measurement class (brick:Relative_Humidity_Sensor / brick:Temperature_Sensor), brick:isPartOf entity:HVAC, with its timeseries and unit, but NO rec:locatedIn</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Client directed: treat as orphans like the register-absent units, do not assume they belong to the register CCUs that share those rooms. The tag is the sensor itself, so it is the point; its equipment parent is unknown, so only HVAC-system membership is asserted.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>

</xml_diff>